<commit_message>
Mark Etsy/Amazon/Daraz listings as own channels; record backlink work
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0113gRVoUz4VftuEgMt9wVK3
</commit_message>
<xml_diff>
--- a/Kordovan_Backlink_Prospects.xlsx
+++ b/Kordovan_Backlink_Prospects.xlsx
@@ -1198,166 +1198,166 @@
       <c r="L13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Is this ours?</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Own channel (live)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Etsy: KordovanLeatherUS (Delaware, US)</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>https://www.etsy.com/uk/shop/KordovanLeatherUS</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Shop named 'Kordovan Leather', also sells 'ILLUSION // Magic Wallet by Kordovan'.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Ours and still live. Add kordovanleather.com wherever Etsy allows it (shop About section), and make sure the shop name and photos match the current brand.</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Etsy shop manager</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Own channel (inactive)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Amazon.ae: 'Kordovan Horse Long Wallet - Maroon'</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ae/Kordovan-Horse-Long-Wallet-Maroon/dp/B098B5T217</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Listing using the Kordovan name in the UAE.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>If it's yours: add the website link. If not: someone is using the brand name. Report it to Etsy.</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>You check</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Ours, inactive. Nothing needed for links. If the seller account still opens, delist the old listings so brand searches don't land on unavailable products.</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Seller account, if still accessible</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Is this ours?</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Amazon.ae: 'Kordovan Horse Long Wallet - Maroon'</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>https://www.amazon.ae/Kordovan-Horse-Long-Wallet-Maroon/dp/B098B5T217</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Listing using the Kordovan name in the UAE.</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Own channel (inactive)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Daraz: 'Kordvan - Smart KODO Wallet' and 'Kordovan Leather' laptop bags</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://www.daraz.pk/products/kordvan-smart-kodo-wallet-wallet-for-men-made-with-horse-leather-card-holde</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Daraz listings with the brand name (one misspelt 'Kordvan'). Rank for brand searches.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Same as above.</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>You check</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>No (Daraz doesn't allow)</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Ours, inactive. Nothing needed for links. If the seller account still opens, delist the old listings so brand searches don't land on unavailable products.</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>Seller account, if still accessible</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Verify</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Is this ours?</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Daraz: 'Kordvan - Smart KODO Wallet' and 'Kordovan Leather' laptop bags</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>https://www.daraz.pk/products/kordvan-smart-kodo-wallet-wallet-for-men-made-with-horse-leather-card-holde</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Daraz listings with the brand name (one misspelt 'Kordvan'). Rank for brand searches.</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>No (Daraz doesn't allow)</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>If yours: fix the spelling to Kordovan so brand searches match. If not: report to Daraz.</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>You check</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr"/>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">

</xml_diff>